<commit_message>
Memperbaiki kesalahan kecil di Analisa
</commit_message>
<xml_diff>
--- a/data/Analisis_Peserta_71261259.xlsx
+++ b/data/Analisis_Peserta_71261259.xlsx
@@ -5,29 +5,24 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\UTS_IT0022_71261259\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64E68309-231B-429E-B204-24A237B53FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E7BBE1C-0917-4645-B859-DF8461EE480B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{F50A1EEF-7038-4FFD-8C2C-A63D5BA7C66B}"/>
+    <workbookView xWindow="0" yWindow="4185" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{F50A1EEF-7038-4FFD-8C2C-A63D5BA7C66B}"/>
   </bookViews>
   <sheets>
     <sheet name="Data_Mentah" sheetId="1" r:id="rId1"/>
     <sheet name="Data_Bersih" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">Data_Bersih!$I$31</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">Data_Bersih!$L$2:$L$27</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">Data_Bersih!$N$27</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">Data_Bersih!$N$2:$N$26</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">Data_Bersih!$I$31</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">Data_Bersih!$L$2:$L$27</definedName>
+    <definedName name="_xlchart.v1.0" hidden="1">Data_Bersih!$L$2:$L$27</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="19" r:id="rId3"/>
-    <pivotCache cacheId="27" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
+    <pivotCache cacheId="1" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -318,9 +313,6 @@
     <t>Kemampuan Belajar</t>
   </si>
   <si>
-    <t>2. Banyak mahasiswa yang mengalami peningkatan nilai setelah mendapat materi, terlihat dari perbedaan nilai pretest dan posttest</t>
-  </si>
-  <si>
     <t>Lulus</t>
   </si>
   <si>
@@ -333,7 +325,10 @@
     <t>3. Disarankan mahasiswa Sistem Informasi diberikan pembinaan mengenai cara belajar yang baik dan efektif, melihat dari jumlah mahasiswa yang tidak lulus</t>
   </si>
   <si>
-    <t>Penemuan:</t>
+    <t>2. Banyak mahasiswa yang mengalami peningkatan nilai setelah mendapat materi, terlihat dari perbedaan nilai pretest dan post test</t>
+  </si>
+  <si>
+    <t>Penemuan yang didapat:</t>
   </si>
 </sst>
 </file>
@@ -432,7 +427,7 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -935,6 +930,11 @@
                 </a:contourClr>
               </a:sp3d>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-9EA7-4B92-ACB1-EBA732C6F041}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -958,6 +958,11 @@
                 </a:contourClr>
               </a:sp3d>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-9EA7-4B92-ACB1-EBA732C6F041}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -981,6 +986,11 @@
                 </a:contourClr>
               </a:sp3d>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-9EA7-4B92-ACB1-EBA732C6F041}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
             <c:spPr>
@@ -1170,7 +1180,7 @@
   <cx:chartData>
     <cx:data id="0">
       <cx:numDim type="val">
-        <cx:f>_xlchart.v1.1</cx:f>
+        <cx:f>_xlchart.v1.0</cx:f>
       </cx:numDim>
     </cx:data>
   </cx:chartData>
@@ -2380,8 +2390,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6562725" y="5891212"/>
-              <a:ext cx="4676775" cy="2743200"/>
+              <a:off x="7124700" y="5891212"/>
+              <a:ext cx="5105400" cy="2743200"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -3433,93 +3443,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CE71A6F6-B147-43C4-B487-7F66B831F926}" name="PivotTable4" cacheId="27" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="B58:E65" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="14">
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="3"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="9" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisCol" dataField="1" showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="10" showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="10"/>
-  </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of Status Sertifikat" fld="10" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FF2BE619-02CC-4CDF-86FF-017F7992E730}" name="PivotTable2" cacheId="19" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{FF2BE619-02CC-4CDF-86FF-017F7992E730}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="B31:F56" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="13">
     <pivotField showAll="0"/>
@@ -3694,6 +3618,92 @@
   </colItems>
   <dataFields count="1">
     <dataField name="Count of Keterangan" fld="12" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{CE71A6F6-B147-43C4-B487-7F66B831F926}" name="PivotTable4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="B58:E65" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <pivotFields count="14">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="3"/>
+        <item x="4"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="9" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" dataField="1" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="10" showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="10"/>
+  </colFields>
+  <colItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Status Sertifikat" fld="10" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -6607,13 +6617,13 @@
     </row>
     <row r="58" spans="2:14" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B58" s="3" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C58" s="3" t="s">
         <v>85</v>
       </c>
       <c r="N58" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="59" spans="2:14" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6621,16 +6631,16 @@
         <v>77</v>
       </c>
       <c r="C59" t="s">
+        <v>88</v>
+      </c>
+      <c r="D59" t="s">
         <v>89</v>
-      </c>
-      <c r="D59" t="s">
-        <v>90</v>
       </c>
       <c r="E59" t="s">
         <v>78</v>
       </c>
       <c r="N59" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="60" spans="2:14" x14ac:dyDescent="0.25">

</xml_diff>